<commit_message>
began av bay cad
</commit_message>
<xml_diff>
--- a/FC_BOM_1.xlsx
+++ b/FC_BOM_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\murth099\Documents\GitHub\FalseConfidence\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owenm\OneDrive\Documents\GitHub\FalseConfidence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14CB8BB5-2A72-4881-9F13-6CB7166BFD41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{013E052B-1478-4269-8E2D-D1268A915BD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{0F8B7B90-5A58-4669-B024-8182CB888A0D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0F8B7B90-5A58-4669-B024-8182CB888A0D}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials" sheetId="1" r:id="rId1"/>
@@ -28,17 +28,16 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="103">
   <si>
     <t>Part Number</t>
   </si>
@@ -175,9 +174,6 @@
     <t>May need more/less idk</t>
   </si>
   <si>
-    <t>LiPos</t>
-  </si>
-  <si>
     <t>Power Switch</t>
   </si>
   <si>
@@ -332,6 +328,24 @@
   </si>
   <si>
     <t>Sustainer &amp; Booster Drogue Chute</t>
+  </si>
+  <si>
+    <t>1s 500mAh LiPo</t>
+  </si>
+  <si>
+    <t>2s 550mAh LiPo</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/OVONIC-Battery-Package-Including-Batteries/dp/B0D3F67LVM/ref=sxin_17_pa_sp_search_thematic_sspa?content-id=amzn1.sym.06dae8e6-5073-49f2-9bdc-0faebb40a382%3Aamzn1.sym.06dae8e6-5073-49f2-9bdc-0faebb40a382&amp;crid=26XR47UAI01E7&amp;cv_ct_cx=1s+lipo&amp;keywords=1s+lipo&amp;pd_rd_i=B0D3F67LVM&amp;pd_rd_r=f5934ac5-da9d-4f88-b8d0-e9c70f0612ad&amp;pd_rd_w=PwlSi&amp;pd_rd_wg=zjobM&amp;pf_rd_p=06dae8e6-5073-49f2-9bdc-0faebb40a382&amp;pf_rd_r=C22DXJ0ZPSD34RPSWM57&amp;qid=1779561723&amp;sbo=RZvfv%2F%2FHxDF%2BO5021pAnSA%3D%3D&amp;sprefix=1s+lipo%2Caps%2C170&amp;sr=1-3-9630ce6b-eb04-480e-8729-567d2ef7dacb-spons&amp;aref=HfagKria8m&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9zZWFyY2hfdGhlbWF0aWM&amp;psc=1</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/OVONIC-7-4V-100C-550mAh-Battery/dp/B0D3F64G3V/ref=sr_1_2_sspa?crid=1Q9OHNBUT6Y5J&amp;dib=eyJ2IjoiMSJ9.xdPVLGAuBS2vf0oiToa5H9WZufPob75J1pUXmhOzrQxYs1EQ1kc1BUHTPUat4HPzZ8eN0rU3rD4NH04V-b4ycGE30pzMTTZWmIiTRcIZrH9NVEqVzX91OhuYc006Nx922hVfnTIxdVk3p44xrSBhcOUAomoquMKAglTRwhyQ0jeLalY5MiELxQeb1DtiFh1APPCbK7HVdsID_lEh-THiczlpP7I8Ex123cTVY938TxN3ET7CByT3JHgWOhIWm4Ge2rto0VgwZbBWiMyTYU0jIF6eJMk2u2nMp9IS94owx50.qbfhjiCv0uE_Eaa7koDBLPQRencqiMqDal18uWLDxfc&amp;dib_tag=se&amp;keywords=550mah+2s+lipo&amp;qid=1779561592&amp;sprefix=50mah+2s+lipo%2Caps%2C163&amp;sr=8-2-spons&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1</t>
+  </si>
+  <si>
+    <t>1s 200mAh LiPo</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/Ransanx-Rechargeable-Integrated-Protection-Electronic/dp/B0F37Y7718/ref=sr_1_1?crid=2EYS8AW7XULA0&amp;dib=eyJ2IjoiMSJ9.lwhlIn-3mJAhDlK7ArO9cHJhwZO1UrBcUnC0S37_WY7orp7i4uLcA3x-3X13hr8wbhOFfhNeJso7oTPpzOtuE4I_PEaWWD2zitIllolHtReq6Lb3hmzYBRE3i1FHtwaDXUkmQG3apMwXnAZOyoJTElr-rblVB6Jy_6OEl51Bo043YirU2NXOgTNLJLkvPfzik8YZhhVh85p88b-wM-R-mXeGAfI_KorlUymNy5h0YA0twAuiLP6MfqzZQo5pBFm9PN9W8WqkCjCI512E-CDyxjMDnGzW3PdFOOgmRUiswyY.DUmf9PB-FTZrlbLKVKFtr6T4Wz5nU2uZzFNLpr7GB0o&amp;dib_tag=se&amp;keywords=1s%2Blipo%2B200mah&amp;qid=1779562203&amp;s=electronics&amp;sprefix=1s%2Blipo%2B200mah%2Celectronics%2C142&amp;sr=1-1&amp;th=1</t>
   </si>
 </sst>
 </file>
@@ -422,7 +436,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -441,23 +455,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="44" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="44" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -478,9 +486,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -518,7 +526,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -624,7 +632,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -766,7 +774,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -774,17 +782,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04C54A36-4462-4840-9712-8BFD36A23A15}">
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.140625" customWidth="1"/>
-    <col min="2" max="2" width="21" style="8" customWidth="1"/>
+    <col min="2" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="14.85546875" customWidth="1"/>
     <col min="4" max="4" width="5.28515625" customWidth="1"/>
     <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="12" style="10" customWidth="1"/>
-    <col min="7" max="7" width="12.28515625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="20" style="10" customWidth="1"/>
+    <col min="6" max="6" width="12" style="9" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" style="9" customWidth="1"/>
+    <col min="8" max="8" width="20" style="9" customWidth="1"/>
     <col min="9" max="9" width="58.140625" customWidth="1"/>
     <col min="11" max="11" width="21.5703125" customWidth="1"/>
   </cols>
@@ -805,13 +813,13 @@
       <c r="E1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="8" t="s">
         <v>27</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -822,24 +830,24 @@
       </c>
     </row>
     <row r="2" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
+      <c r="A2" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
       <c r="K2" s="5"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" t="s">
         <v>33</v>
       </c>
       <c r="C3">
@@ -851,27 +859,27 @@
       <c r="E3">
         <v>1</v>
       </c>
-      <c r="F3" s="10">
+      <c r="F3" s="9">
         <v>175</v>
       </c>
-      <c r="G3" s="10">
+      <c r="G3" s="9">
         <f>E3*F3</f>
         <v>175</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="9">
         <f>(E3-C3)*F3</f>
         <v>175</v>
       </c>
       <c r="K3" s="6">
         <f>SUM(G:G)</f>
-        <v>1654.5700000000002</v>
+        <v>1689.5400000000002</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" t="s">
         <v>34</v>
       </c>
       <c r="C4">
@@ -883,15 +891,15 @@
       <c r="E4">
         <v>1</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="9">
         <v>80</v>
       </c>
-      <c r="G4" s="10">
-        <f t="shared" ref="G4:G56" si="0">E4*F4</f>
+      <c r="G4" s="9">
+        <f t="shared" ref="G4:G58" si="0">E4*F4</f>
         <v>80</v>
       </c>
-      <c r="H4" s="10">
-        <f t="shared" ref="H4:H56" si="1">(E4-C4)*F4</f>
+      <c r="H4" s="9">
+        <f t="shared" ref="H4:H58" si="1">(E4-C4)*F4</f>
         <v>80</v>
       </c>
       <c r="K4" s="5" t="s">
@@ -902,7 +910,7 @@
       <c r="A5" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" t="s">
         <v>29</v>
       </c>
       <c r="C5">
@@ -914,27 +922,27 @@
       <c r="E5">
         <v>1</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="9">
         <v>170</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="9">
         <f t="shared" si="0"/>
         <v>170</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="9">
         <f t="shared" si="1"/>
         <v>170</v>
       </c>
       <c r="K5" s="7">
         <f>SUM(H:H)</f>
-        <v>1263.4599999999998</v>
+        <v>1285.4399999999998</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" t="s">
         <v>29</v>
       </c>
       <c r="C6">
@@ -946,106 +954,106 @@
       <c r="E6">
         <v>1</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="9">
         <v>195</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="9">
         <f t="shared" si="0"/>
         <v>195</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="9">
         <f t="shared" si="1"/>
         <v>195</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10">
+        <v>0</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="10">
+        <v>1</v>
+      </c>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H7" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="11">
-        <v>0</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="11">
-        <v>1</v>
-      </c>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H7" s="13">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B8" s="12"/>
-      <c r="C8" s="11">
-        <v>0</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="11">
-        <v>1</v>
-      </c>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H8" s="13">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I8" s="11" t="s">
-        <v>49</v>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10">
+        <v>0</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="10">
+        <v>1</v>
+      </c>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H8" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="11">
-        <v>0</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="11">
+      <c r="C9" s="10">
+        <v>0</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="10">
         <v>2</v>
       </c>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H9" s="13">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I9" s="11" t="s">
-        <v>49</v>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H9" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" t="s">
         <v>40</v>
       </c>
       <c r="C10">
@@ -1057,14 +1065,14 @@
       <c r="E10">
         <v>1</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="9">
         <v>100</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="9">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1073,7 +1081,7 @@
       <c r="A11" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" t="s">
         <v>40</v>
       </c>
       <c r="C11">
@@ -1085,14 +1093,14 @@
       <c r="E11">
         <v>1</v>
       </c>
-      <c r="F11" s="10">
+      <c r="F11" s="9">
         <v>20</v>
       </c>
-      <c r="G11" s="10">
+      <c r="G11" s="9">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="H11" s="10">
+      <c r="H11" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1101,7 +1109,7 @@
       <c r="A12" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" t="s">
         <v>40</v>
       </c>
       <c r="C12">
@@ -1113,14 +1121,14 @@
       <c r="E12">
         <v>1</v>
       </c>
-      <c r="F12" s="10">
+      <c r="F12" s="9">
         <v>55</v>
       </c>
-      <c r="G12" s="10">
+      <c r="G12" s="9">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
-      <c r="H12" s="10">
+      <c r="H12" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1129,7 +1137,7 @@
       <c r="A13" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" t="s">
         <v>42</v>
       </c>
       <c r="C13">
@@ -1141,354 +1149,362 @@
       <c r="E13">
         <v>1</v>
       </c>
-      <c r="F13" s="10">
+      <c r="F13" s="9">
         <v>82.99</v>
       </c>
-      <c r="G13" s="10">
+      <c r="G13" s="9">
         <f t="shared" si="0"/>
         <v>82.99</v>
       </c>
-      <c r="H13" s="10">
+      <c r="H13" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" s="11"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H14" s="13">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I14" s="11" t="s">
-        <v>49</v>
+      <c r="A14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B14" t="s">
+        <v>102</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14" s="9">
+        <v>10.99</v>
+      </c>
+      <c r="G14" s="9">
+        <f t="shared" si="0"/>
+        <v>10.99</v>
+      </c>
+      <c r="H14" s="9">
+        <f t="shared" si="1"/>
+        <v>10.99</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>97</v>
+      </c>
+      <c r="B15" t="s">
+        <v>99</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15" s="9">
+        <v>10.99</v>
+      </c>
+      <c r="G15" s="9">
+        <f t="shared" si="0"/>
+        <v>10.99</v>
+      </c>
+      <c r="H15" s="9">
+        <f t="shared" si="1"/>
+        <v>10.99</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" t="s">
+        <v>100</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16" s="9">
+        <v>12.99</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="0"/>
+        <v>12.99</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I16" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17">
+        <v>6</v>
+      </c>
+      <c r="F17" s="9">
+        <v>8.5</v>
+      </c>
+      <c r="G17" s="9">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+      <c r="H17" s="9">
+        <f t="shared" si="1"/>
+        <v>42.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="C15">
-        <v>1</v>
-      </c>
-      <c r="D15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E15">
-        <v>6</v>
-      </c>
-      <c r="F15" s="10">
-        <v>8.5</v>
-      </c>
-      <c r="G15" s="10">
-        <f t="shared" si="0"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" s="10"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H18" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20" s="9">
+        <v>42</v>
+      </c>
+      <c r="G20" s="9">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="H20" s="9">
+        <f t="shared" si="1"/>
+        <v>42</v>
+      </c>
+      <c r="I20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>66</v>
+      </c>
+      <c r="B21" t="s">
         <v>51</v>
       </c>
-      <c r="H15" s="10">
-        <f t="shared" si="1"/>
-        <v>42.5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="B16" s="12"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E16" s="11"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H16" s="13">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I16" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>69</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-      <c r="D18" t="s">
-        <v>13</v>
-      </c>
-      <c r="E18">
-        <v>1</v>
-      </c>
-      <c r="F18" s="10">
-        <v>42</v>
-      </c>
-      <c r="G18" s="10">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="H18" s="10">
-        <f t="shared" si="1"/>
-        <v>42</v>
-      </c>
-      <c r="I18" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21" s="9">
+        <v>26.55</v>
+      </c>
+      <c r="G21" s="9">
+        <f t="shared" si="0"/>
+        <v>26.55</v>
+      </c>
+      <c r="H21" s="9">
+        <f t="shared" si="1"/>
+        <v>26.55</v>
+      </c>
+      <c r="I21" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10">
+        <v>0</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" s="10">
+        <v>1</v>
+      </c>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H22" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I22" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10">
+        <v>0</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" s="10">
+        <v>1</v>
+      </c>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H23" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I23" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B24" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24" s="9">
+        <v>7.11</v>
+      </c>
+      <c r="G24" s="9">
+        <f t="shared" si="0"/>
+        <v>7.11</v>
+      </c>
+      <c r="H24" s="9">
+        <f t="shared" si="1"/>
+        <v>7.11</v>
+      </c>
+      <c r="I24" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="14">
-        <v>0</v>
-      </c>
-      <c r="D19" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" s="14">
-        <v>1</v>
-      </c>
-      <c r="F19" s="10">
-        <v>26.55</v>
-      </c>
-      <c r="G19" s="10">
-        <f t="shared" si="0"/>
-        <v>26.55</v>
-      </c>
-      <c r="H19" s="10">
-        <f t="shared" si="1"/>
-        <v>26.55</v>
-      </c>
-      <c r="I19" s="14" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B20" s="12"/>
-      <c r="C20" s="11">
-        <v>0</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E20" s="11">
-        <v>1</v>
-      </c>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H20" s="13">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I20" s="11" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="11">
-        <v>0</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E21" s="11">
-        <v>1</v>
-      </c>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H21" s="13">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I21" s="11" t="s">
+      <c r="B25" s="10"/>
+      <c r="C25" s="10">
+        <v>0</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E25" s="10">
+        <v>1</v>
+      </c>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H25" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I25" s="10" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22" t="s">
-        <v>13</v>
-      </c>
-      <c r="E22">
-        <v>1</v>
-      </c>
-      <c r="F22" s="10">
-        <v>7.11</v>
-      </c>
-      <c r="G22" s="10">
-        <f t="shared" si="0"/>
-        <v>7.11</v>
-      </c>
-      <c r="H22" s="10">
-        <f t="shared" si="1"/>
-        <v>7.11</v>
-      </c>
-      <c r="I22" s="14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="11">
-        <v>0</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E23" s="11">
-        <v>1</v>
-      </c>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H23" s="13">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I23" s="11" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
-      <c r="I24" s="15"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C25">
-        <v>0</v>
-      </c>
-      <c r="D25" t="s">
-        <v>13</v>
-      </c>
-      <c r="E25">
-        <v>1</v>
-      </c>
-      <c r="F25" s="10">
-        <v>7.88</v>
-      </c>
-      <c r="G25" s="10">
-        <f t="shared" si="0"/>
-        <v>7.88</v>
-      </c>
-      <c r="H25" s="10">
-        <f t="shared" si="1"/>
-        <v>7.88</v>
-      </c>
-    </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>66</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-      <c r="D26" t="s">
-        <v>13</v>
-      </c>
-      <c r="E26">
-        <v>1</v>
-      </c>
-      <c r="F26" s="10">
-        <v>15.51</v>
-      </c>
-      <c r="G26" s="10">
-        <f t="shared" si="0"/>
-        <v>15.51</v>
-      </c>
-      <c r="H26" s="10">
-        <f t="shared" si="1"/>
-        <v>15.51</v>
-      </c>
+      <c r="A26" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>65</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
+      </c>
+      <c r="B27" t="s">
+        <v>59</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -1499,24 +1515,24 @@
       <c r="E27">
         <v>1</v>
       </c>
-      <c r="F27" s="10">
-        <v>12.63</v>
-      </c>
-      <c r="G27" s="10">
-        <f t="shared" si="0"/>
-        <v>12.63</v>
-      </c>
-      <c r="H27" s="10">
-        <f t="shared" si="1"/>
-        <v>12.63</v>
+      <c r="F27" s="9">
+        <v>7.88</v>
+      </c>
+      <c r="G27" s="9">
+        <f t="shared" si="0"/>
+        <v>7.88</v>
+      </c>
+      <c r="H27" s="9">
+        <f t="shared" si="1"/>
+        <v>7.88</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>71</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>73</v>
+        <v>65</v>
+      </c>
+      <c r="B28" t="s">
+        <v>63</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -1525,29 +1541,29 @@
         <v>13</v>
       </c>
       <c r="E28">
-        <v>2</v>
-      </c>
-      <c r="F28" s="10">
-        <v>3.65</v>
-      </c>
-      <c r="G28" s="10">
-        <f t="shared" si="0"/>
-        <v>7.3</v>
-      </c>
-      <c r="H28" s="10">
-        <f t="shared" si="1"/>
-        <v>7.3</v>
+        <v>1</v>
+      </c>
+      <c r="F28" s="9">
+        <v>15.51</v>
+      </c>
+      <c r="G28" s="9">
+        <f t="shared" si="0"/>
+        <v>15.51</v>
+      </c>
+      <c r="H28" s="9">
+        <f t="shared" si="1"/>
+        <v>15.51</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>74</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>75</v>
+        <v>64</v>
+      </c>
+      <c r="B29" t="s">
+        <v>69</v>
       </c>
       <c r="C29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" t="s">
         <v>13</v>
@@ -1555,195 +1571,189 @@
       <c r="E29">
         <v>1</v>
       </c>
-      <c r="F29" s="10">
-        <v>10.67</v>
-      </c>
-      <c r="G29" s="10">
-        <f t="shared" si="0"/>
-        <v>10.67</v>
-      </c>
-      <c r="H29" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+      <c r="F29" s="9">
+        <v>12.63</v>
+      </c>
+      <c r="G29" s="9">
+        <f t="shared" si="0"/>
+        <v>12.63</v>
+      </c>
+      <c r="H29" s="9">
+        <f t="shared" si="1"/>
+        <v>12.63</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" t="s">
+        <v>72</v>
+      </c>
+      <c r="C30">
+        <v>0</v>
+      </c>
+      <c r="D30" t="s">
+        <v>13</v>
+      </c>
+      <c r="E30">
+        <v>2</v>
+      </c>
+      <c r="F30" s="9">
+        <v>3.65</v>
+      </c>
+      <c r="G30" s="9">
+        <f t="shared" si="0"/>
+        <v>7.3</v>
+      </c>
+      <c r="H30" s="9">
+        <f t="shared" si="1"/>
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>73</v>
+      </c>
+      <c r="B31" t="s">
+        <v>74</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+      <c r="D31" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="F31" s="9">
+        <v>10.67</v>
+      </c>
+      <c r="G31" s="9">
+        <f t="shared" si="0"/>
+        <v>10.67</v>
+      </c>
+      <c r="H31" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>75</v>
+      </c>
+      <c r="B32" t="s">
         <v>76</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="C32">
+        <v>1</v>
+      </c>
+      <c r="D32" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32" s="9">
+        <v>5.5</v>
+      </c>
+      <c r="G32" s="9">
+        <f t="shared" si="0"/>
+        <v>5.5</v>
+      </c>
+      <c r="H32" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="C30">
-        <v>1</v>
-      </c>
-      <c r="D30" t="s">
-        <v>13</v>
-      </c>
-      <c r="E30">
-        <v>1</v>
-      </c>
-      <c r="F30" s="10">
-        <v>5.5</v>
-      </c>
-      <c r="G30" s="10">
-        <f t="shared" si="0"/>
-        <v>5.5</v>
-      </c>
-      <c r="H30" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="17" t="s">
+      <c r="B33" s="12"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="12"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="10"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" s="10"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H34" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I34" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="17"/>
-      <c r="I31" s="17"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="11"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E32" s="11"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H32" s="13">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I32" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="17" t="s">
+      <c r="B35" s="12"/>
+      <c r="C35" s="12"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="12"/>
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="12"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="10"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36" s="10"/>
+      <c r="F36" s="11"/>
+      <c r="G36" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H36" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I36" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="17"/>
-      <c r="I33" s="17"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="11"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E34" s="11"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H34" s="13">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I34" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="17"/>
-      <c r="G35" s="17"/>
-      <c r="H35" s="17"/>
-      <c r="I35" s="17"/>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>81</v>
-      </c>
-      <c r="B36" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C36">
-        <v>0</v>
-      </c>
-      <c r="D36" t="s">
-        <v>13</v>
-      </c>
-      <c r="E36">
-        <v>1</v>
-      </c>
-      <c r="F36" s="10">
-        <v>269.99</v>
-      </c>
-      <c r="G36" s="10">
-        <f t="shared" si="0"/>
-        <v>269.99</v>
-      </c>
-      <c r="H36" s="10">
-        <f t="shared" si="1"/>
-        <v>269.99</v>
-      </c>
-      <c r="I36" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>82</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C37">
-        <v>0</v>
-      </c>
-      <c r="D37" t="s">
-        <v>13</v>
-      </c>
-      <c r="E37">
-        <v>1</v>
-      </c>
-      <c r="F37" s="10">
-        <v>167.99</v>
-      </c>
-      <c r="G37" s="10">
-        <f t="shared" si="0"/>
-        <v>167.99</v>
-      </c>
-      <c r="H37" s="10">
-        <f t="shared" si="1"/>
-        <v>167.99</v>
-      </c>
-      <c r="I37" t="s">
-        <v>83</v>
-      </c>
+      <c r="B37" s="12"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="12"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>85</v>
-      </c>
-      <c r="B38" s="8" t="s">
-        <v>86</v>
+        <v>80</v>
+      </c>
+      <c r="B38" t="s">
+        <v>48</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -1752,29 +1762,32 @@
         <v>13</v>
       </c>
       <c r="E38">
-        <v>2</v>
-      </c>
-      <c r="F38" s="10">
-        <v>16</v>
-      </c>
-      <c r="G38" s="10">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-      <c r="H38" s="10">
-        <f t="shared" si="1"/>
-        <v>32</v>
+        <v>1</v>
+      </c>
+      <c r="F38" s="9">
+        <v>269.99</v>
+      </c>
+      <c r="G38" s="9">
+        <f t="shared" si="0"/>
+        <v>269.99</v>
+      </c>
+      <c r="H38" s="9">
+        <f t="shared" si="1"/>
+        <v>269.99</v>
+      </c>
+      <c r="I38" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>87</v>
-      </c>
-      <c r="B39" s="8" t="s">
-        <v>88</v>
+        <v>81</v>
+      </c>
+      <c r="B39" t="s">
+        <v>48</v>
       </c>
       <c r="C39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D39" t="s">
         <v>13</v>
@@ -1782,55 +1795,55 @@
       <c r="E39">
         <v>1</v>
       </c>
-      <c r="F39" s="10">
-        <v>38</v>
-      </c>
-      <c r="G39" s="10">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-      <c r="H39" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+      <c r="F39" s="9">
+        <v>167.99</v>
+      </c>
+      <c r="G39" s="9">
+        <f t="shared" si="0"/>
+        <v>167.99</v>
+      </c>
+      <c r="H39" s="9">
+        <f t="shared" si="1"/>
+        <v>167.99</v>
+      </c>
+      <c r="I39" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>89</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>92</v>
+        <v>84</v>
+      </c>
+      <c r="B40" t="s">
+        <v>85</v>
       </c>
       <c r="C40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D40" t="s">
         <v>13</v>
       </c>
       <c r="E40">
-        <v>1</v>
-      </c>
-      <c r="F40" s="10">
-        <v>34.5</v>
-      </c>
-      <c r="G40" s="10">
-        <f>E40*F40</f>
-        <v>34.5</v>
-      </c>
-      <c r="H40" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I40" t="s">
-        <v>95</v>
+        <v>2</v>
+      </c>
+      <c r="F40" s="9">
+        <v>16</v>
+      </c>
+      <c r="G40" s="9">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="H40" s="9">
+        <f t="shared" si="1"/>
+        <v>32</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>93</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>94</v>
+        <v>86</v>
+      </c>
+      <c r="B41" t="s">
+        <v>87</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -1841,87 +1854,120 @@
       <c r="E41">
         <v>1</v>
       </c>
-      <c r="F41" s="10">
-        <v>35.950000000000003</v>
-      </c>
-      <c r="G41" s="10">
-        <f>E41*F41</f>
-        <v>35.950000000000003</v>
-      </c>
-      <c r="H41" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I41" t="s">
-        <v>96</v>
+      <c r="F41" s="9">
+        <v>38</v>
+      </c>
+      <c r="G41" s="9">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="H41" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>88</v>
+      </c>
+      <c r="B42" t="s">
+        <v>91</v>
+      </c>
+      <c r="C42">
+        <v>1</v>
+      </c>
+      <c r="D42" t="s">
+        <v>13</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+      <c r="F42" s="9">
+        <v>34.5</v>
+      </c>
+      <c r="G42" s="9">
+        <f>E42*F42</f>
+        <v>34.5</v>
+      </c>
+      <c r="H42" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I42" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>92</v>
+      </c>
+      <c r="B43" t="s">
+        <v>93</v>
+      </c>
+      <c r="C43">
+        <v>1</v>
+      </c>
+      <c r="D43" t="s">
+        <v>13</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="F43" s="9">
+        <v>35.950000000000003</v>
+      </c>
+      <c r="G43" s="9">
+        <f>E43*F43</f>
+        <v>35.950000000000003</v>
+      </c>
+      <c r="H43" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I43" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>89</v>
+      </c>
+      <c r="B44" t="s">
         <v>90</v>
       </c>
-      <c r="B42" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="C42">
-        <v>0</v>
-      </c>
-      <c r="D42" t="s">
-        <v>13</v>
-      </c>
-      <c r="E42">
+      <c r="C44">
+        <v>0</v>
+      </c>
+      <c r="D44" t="s">
+        <v>13</v>
+      </c>
+      <c r="E44">
         <v>2</v>
       </c>
-      <c r="F42" s="10">
+      <c r="F44" s="9">
         <v>6</v>
       </c>
-      <c r="G42" s="10">
-        <f>E42*F42</f>
+      <c r="G44" s="9">
+        <f>E44*F44</f>
         <v>12</v>
       </c>
-      <c r="H42" s="10">
-        <f>(E42-C42)*F42</f>
+      <c r="H44" s="9">
+        <f>(E44-C44)*F44</f>
         <v>12</v>
       </c>
-      <c r="I42" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D43" t="s">
-        <v>13</v>
-      </c>
-      <c r="G43" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H43" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D44" t="s">
-        <v>13</v>
-      </c>
-      <c r="G44" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H44" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+      <c r="I44" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D45" t="s">
         <v>13</v>
       </c>
-      <c r="G45" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H45" s="10">
+      <c r="G45" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H45" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1930,11 +1976,11 @@
       <c r="D46" t="s">
         <v>13</v>
       </c>
-      <c r="G46" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H46" s="10">
+      <c r="G46" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H46" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1943,11 +1989,11 @@
       <c r="D47" t="s">
         <v>13</v>
       </c>
-      <c r="G47" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H47" s="10">
+      <c r="G47" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H47" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1956,11 +2002,11 @@
       <c r="D48" t="s">
         <v>13</v>
       </c>
-      <c r="G48" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H48" s="10">
+      <c r="G48" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H48" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1969,11 +2015,11 @@
       <c r="D49" t="s">
         <v>13</v>
       </c>
-      <c r="G49" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H49" s="10">
+      <c r="G49" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H49" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1982,11 +2028,11 @@
       <c r="D50" t="s">
         <v>13</v>
       </c>
-      <c r="G50" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H50" s="10">
+      <c r="G50" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H50" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1995,11 +2041,11 @@
       <c r="D51" t="s">
         <v>13</v>
       </c>
-      <c r="G51" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H51" s="10">
+      <c r="G51" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H51" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2008,11 +2054,11 @@
       <c r="D52" t="s">
         <v>13</v>
       </c>
-      <c r="G52" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H52" s="10">
+      <c r="G52" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H52" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2021,11 +2067,11 @@
       <c r="D53" t="s">
         <v>13</v>
       </c>
-      <c r="G53" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H53" s="10">
+      <c r="G53" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H53" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2034,11 +2080,11 @@
       <c r="D54" t="s">
         <v>13</v>
       </c>
-      <c r="G54" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H54" s="10">
+      <c r="G54" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H54" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2047,11 +2093,11 @@
       <c r="D55" t="s">
         <v>13</v>
       </c>
-      <c r="G55" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H55" s="10">
+      <c r="G55" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H55" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2060,21 +2106,47 @@
       <c r="D56" t="s">
         <v>13</v>
       </c>
-      <c r="G56" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H56" s="10">
+      <c r="G56" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H56" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G57" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H57" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D58" t="s">
+        <v>13</v>
+      </c>
+      <c r="G58" s="9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H58" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A37:I37"/>
+    <mergeCell ref="A19:I19"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A24:I24"/>
-    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A26:I26"/>
     <mergeCell ref="A33:I33"/>
     <mergeCell ref="A35:I35"/>
   </mergeCells>

</xml_diff>